<commit_message>
Corrida | GSF-TD | 2026-10-14 11:14:35.606495
</commit_message>
<xml_diff>
--- a/indicadores/GSF-TD_out.xlsx
+++ b/indicadores/GSF-TD_out.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Porcentaje de despidos</t>
+    <t xml:space="preserve">Porcentaje de despidos en relación al empleo total</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | GSF-TD | 2026-10-14 11:39:44.858612
</commit_message>
<xml_diff>
--- a/indicadores/GSF-TD_out.xlsx
+++ b/indicadores/GSF-TD_out.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Porcentaje de despidos en relación al empleo total</t>
+    <t xml:space="preserve">% de despidos en relación al empleo total</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>